<commit_message>
Expose cohort controls and preserve all saved summary variants
</commit_message>
<xml_diff>
--- a/summary/yes/exposures_meta_analysis_bladder_cancer_combined.xlsx
+++ b/summary/yes/exposures_meta_analysis_bladder_cancer_combined.xlsx
@@ -23,13 +23,16 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -49,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -57,13 +60,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -452,57 +464,57 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Exposure</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>number estimates</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Pooled RR</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>lower CI RR</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>upper CI RR</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>lower PI RR</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>upper PI RR</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>I^2 (%)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>eggers p-value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>total N</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>total Cases</t>
         </is>
@@ -514,26 +526,26 @@
           <t>zeaxanthin</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="n">
+      <c r="B2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>0.1606125118752876</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="4" t="n">
         <v>0.02008938167695712</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="4" t="n">
         <v>1.059711334632446</v>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="5" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr"/>
+      <c r="J2" s="3" t="n">
         <v>257</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="3" t="n">
         <v>84</v>
       </c>
     </row>
@@ -543,26 +555,26 @@
           <t>alpha_linolenic_acid</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="B3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>0.2608764404894685</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="4" t="n">
         <v>0.1004102763893268</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="4" t="n">
         <v>0.6510344938106651</v>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="3" t="n">
         <v>561</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="3" t="n">
         <v>322</v>
       </c>
     </row>
@@ -572,28 +584,28 @@
           <t>omega_3_fatty_acids</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="4" t="n">
         <v>0.3063889211181519</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>0.1968132439764496</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>0.4770185022795724</v>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="4" t="n">
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="3" t="n">
         <v>1061</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="3" t="n">
         <v>572</v>
       </c>
     </row>
@@ -603,26 +615,26 @@
           <t>eicosapentaenoic_acid</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3" t="n">
+      <c r="B5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>0.3209909633019056</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="4" t="n">
         <v>0.19070128490511</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="4" t="n">
         <v>0.5211356588277174</v>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="3" t="n">
         <v>250</v>
       </c>
     </row>
@@ -632,26 +644,26 @@
           <t>docosahexaenoic_acid</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="3" t="n">
+      <c r="B6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>0.331006856656578</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="4" t="n">
         <v>0.20072904790198</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="4" t="n">
         <v>0.5311333323044712</v>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="3" t="n">
         <v>250</v>
       </c>
     </row>
@@ -661,26 +673,26 @@
           <t>multivitamin</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="3" t="n">
+      <c r="B7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>0.3910830654414335</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="4" t="n">
         <v>0.2408309631552709</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="4" t="n">
         <v>0.6310600546798513</v>
       </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="3" t="n">
         <v>667</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="3" t="n">
         <v>262</v>
       </c>
     </row>
@@ -690,28 +702,28 @@
           <t>polyunsaturated_fat_pufa</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="4" t="n">
         <v>0.4049871260142381</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="4" t="n">
         <v>0.2442653853180111</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="4" t="n">
         <v>0.6714605592754802</v>
       </c>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="4" t="n">
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="5" t="n">
         <v>18.64</v>
       </c>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="3" t="n">
         <v>1061</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="3" t="n">
         <v>572</v>
       </c>
     </row>
@@ -721,26 +733,26 @@
           <t>linoleic_acid</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="3" t="n">
+      <c r="B9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>0.4311156410559245</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="4" t="n">
         <v>0.19070128490511</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="4" t="n">
         <v>0.9601743676651679</v>
       </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="3" t="n">
         <v>561</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="3" t="n">
         <v>322</v>
       </c>
     </row>
@@ -750,28 +762,28 @@
           <t>omega_6_fatty_acids</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="4" t="n">
         <v>0.4607498536806614</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="4" t="n">
         <v>0.3074631611655286</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="4" t="n">
         <v>0.6905271414181002</v>
       </c>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="4" t="n">
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="3" t="n">
         <v>1061</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="3" t="n">
         <v>572</v>
       </c>
     </row>
@@ -781,26 +793,26 @@
           <t>dihomo_gamma_linolenic_acid</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="3" t="n">
+      <c r="B11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>0.4711336417688241</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="4" t="n">
         <v>0.2909378089333156</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="4" t="n">
         <v>0.7408745282931972</v>
       </c>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="2" t="n">
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="3" t="n">
         <v>250</v>
       </c>
     </row>
@@ -810,26 +822,26 @@
           <t>olive</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="3" t="n">
+      <c r="B12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>0.4711336417688241</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="4" t="n">
         <v>0.2809182656266805</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="4" t="n">
         <v>0.7807798429070956</v>
       </c>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="3" t="n">
         <v>586</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="3" t="n">
         <v>200</v>
       </c>
     </row>
@@ -839,26 +851,26 @@
           <t>olive_oil_intake</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3" t="n">
+      <c r="B13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>0.4711336417688241</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="4" t="n">
         <v>0.2809182656266805</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="4" t="n">
         <v>0.7807798429070956</v>
       </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="3" t="n">
         <v>586</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="3" t="n">
         <v>200</v>
       </c>
     </row>
@@ -868,26 +880,26 @@
           <t>oleic_acid</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="3" t="n">
+      <c r="B14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>0.54113009609268</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="4" t="n">
         <v>0.3410218378348885</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="4" t="n">
         <v>0.860546963650096</v>
       </c>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="2" t="n">
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="3" t="n">
         <v>250</v>
       </c>
     </row>
@@ -897,26 +909,26 @@
           <t>omega_9_fatty_acids</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="3" t="n">
+      <c r="B15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>0.54113009609268</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="4" t="n">
         <v>0.3410218378348885</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="4" t="n">
         <v>0.860546963650096</v>
       </c>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="3" t="n">
         <v>250</v>
       </c>
     </row>
@@ -926,26 +938,26 @@
           <t>vitamin_b3</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="3" t="n">
+      <c r="B16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="n">
         <v>0.5611208951000519</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="4" t="n">
         <v>0.3109741576462426</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="4" t="n">
         <v>1.019907392408769</v>
       </c>
-      <c r="F16" s="3" t="inlineStr"/>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="3" t="n">
         <v>561</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="3" t="n">
         <v>322</v>
       </c>
     </row>
@@ -955,28 +967,28 @@
           <t>legumes</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="4" t="n">
         <v>0.6397997770084459</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="4" t="n">
         <v>0.4305034246903502</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="4" t="n">
         <v>0.9507539286723269</v>
       </c>
-      <c r="F17" s="3" t="inlineStr"/>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="4" t="n">
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="5" t="n">
         <v>77.91</v>
       </c>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="3" t="n">
         <v>2541</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="K17" s="3" t="n">
         <v>1268</v>
       </c>
     </row>
@@ -986,28 +998,28 @@
           <t>yogurt</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="4" t="n">
         <v>0.6435857533404954</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="4" t="n">
         <v>0.2494242542659014</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="4" t="n">
         <v>1.660634901453039</v>
       </c>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="4" t="n">
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="5" t="n">
         <v>70.34</v>
       </c>
-      <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="3" t="n">
         <v>101981</v>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="K18" s="3" t="n">
         <v>906</v>
       </c>
     </row>
@@ -1017,34 +1029,34 @@
           <t>lutein</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="4" t="n">
         <v>0.6941272346837586</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="4" t="n">
         <v>0.3791588622931857</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="4" t="n">
         <v>1.270740752347649</v>
       </c>
-      <c r="F19" s="3" t="n">
-        <v>0.0007090691841002699</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>679.5001513725188</v>
-      </c>
-      <c r="H19" s="4" t="n">
+      <c r="F19" s="4" t="n">
+        <v>0.0007090691840013509</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>679.5001514673125</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>71.59</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="I19" s="6" t="n">
         <v>0.1894295826083661</v>
       </c>
-      <c r="J19" s="2" t="n">
+      <c r="J19" s="3" t="n">
         <v>122821</v>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="K19" s="3" t="n">
         <v>1415</v>
       </c>
     </row>
@@ -1054,34 +1066,34 @@
           <t>vitamin_a</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="4" t="n">
         <v>0.7164835434120075</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="4" t="n">
         <v>0.5214718421284985</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E20" s="4" t="n">
         <v>0.9843241652031548</v>
       </c>
-      <c r="F20" s="3" t="n">
-        <v>0.2212620745858667</v>
-      </c>
-      <c r="G20" s="3" t="n">
-        <v>2.320093350571054</v>
-      </c>
-      <c r="H20" s="4" t="n">
+      <c r="F20" s="4" t="n">
+        <v>0.2212620745890885</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>2.320093350537271</v>
+      </c>
+      <c r="H20" s="5" t="n">
         <v>46.43</v>
       </c>
-      <c r="I20" s="5" t="n">
-        <v>0.1336757219634318</v>
-      </c>
-      <c r="J20" s="2" t="n">
+      <c r="I20" s="6" t="n">
+        <v>0.1336757219634319</v>
+      </c>
+      <c r="J20" s="3" t="n">
         <v>126541</v>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="K20" s="3" t="n">
         <v>1142</v>
       </c>
     </row>
@@ -1091,34 +1103,34 @@
           <t>whole_grain_intake</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C21" s="4" t="n">
         <v>0.7226718735643111</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="4" t="n">
         <v>0.5177307290339085</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="4" t="n">
         <v>1.008737954989623</v>
       </c>
-      <c r="F21" s="3" t="n">
-        <v>0.01658634469437209</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>31.48702420360033</v>
-      </c>
-      <c r="H21" s="4" t="n">
+      <c r="F21" s="4" t="n">
+        <v>0.01658634469310387</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>31.48702420600785</v>
+      </c>
+      <c r="H21" s="5" t="n">
         <v>75.47</v>
       </c>
-      <c r="I21" s="5" t="n">
-        <v>0.2822678427106021</v>
-      </c>
-      <c r="J21" s="2" t="n">
+      <c r="I21" s="6" t="n">
+        <v>0.282267842710602</v>
+      </c>
+      <c r="J21" s="3" t="n">
         <v>219042</v>
       </c>
-      <c r="K21" s="2" t="n">
+      <c r="K21" s="3" t="n">
         <v>1666</v>
       </c>
     </row>
@@ -1128,34 +1140,34 @@
           <t>selenium</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="4" t="n">
         <v>0.725713478332136</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="4" t="n">
         <v>0.5422110294998878</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E22" s="4" t="n">
         <v>0.9713193276770786</v>
       </c>
-      <c r="F22" s="3" t="n">
-        <v>0.2945606787230922</v>
-      </c>
-      <c r="G22" s="3" t="n">
-        <v>1.787950974705708</v>
-      </c>
-      <c r="H22" s="4" t="n">
+      <c r="F22" s="4" t="n">
+        <v>0.2945606787230932</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>1.787950974705702</v>
+      </c>
+      <c r="H22" s="5" t="n">
         <v>71.62</v>
       </c>
-      <c r="I22" s="5" t="n">
-        <v>0.1356590524221061</v>
-      </c>
-      <c r="J22" s="2" t="n">
+      <c r="I22" s="6" t="n">
+        <v>0.1356590524221063</v>
+      </c>
+      <c r="J22" s="3" t="n">
         <v>161440</v>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="K22" s="3" t="n">
         <v>3121</v>
       </c>
     </row>
@@ -1165,34 +1177,34 @@
           <t>fermented_foods</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B23" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="4" t="n">
         <v>0.7490122054026693</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="4" t="n">
         <v>0.5024294735717695</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="4" t="n">
         <v>1.116613004117546</v>
       </c>
-      <c r="F23" s="3" t="n">
-        <v>0.1999700203677981</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>2.805516961043995</v>
-      </c>
-      <c r="H23" s="4" t="n">
+      <c r="F23" s="4" t="n">
+        <v>0.199970020367752</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>2.805516961044641</v>
+      </c>
+      <c r="H23" s="5" t="n">
         <v>73.37</v>
       </c>
-      <c r="I23" s="5" t="n">
-        <v>0.6646008321307549</v>
-      </c>
-      <c r="J23" s="2" t="n">
+      <c r="I23" s="6" t="n">
+        <v>0.6646008321307553</v>
+      </c>
+      <c r="J23" s="3" t="n">
         <v>203999</v>
       </c>
-      <c r="K23" s="2" t="n">
+      <c r="K23" s="3" t="n">
         <v>2474</v>
       </c>
     </row>
@@ -1202,26 +1214,26 @@
           <t>non_nutritive_sweetener_intake</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="3" t="n">
+      <c r="B24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="n">
         <v>0.7504264322028401</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="4" t="n">
         <v>0.5305667184532947</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="E24" s="4" t="n">
         <v>1.059855422172594</v>
       </c>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="5" t="inlineStr"/>
-      <c r="J24" s="2" t="n">
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="3" t="n">
         <v>80388</v>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="K24" s="3" t="n">
         <v>448</v>
       </c>
     </row>
@@ -1231,34 +1243,34 @@
           <t>vitamin_c</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="4" t="n">
         <v>0.7509621709935039</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="4" t="n">
         <v>0.5556037048097945</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="4" t="n">
         <v>1.014910062303704</v>
       </c>
-      <c r="F25" s="3" t="n">
-        <v>0.05110412975560341</v>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>11.03519783939657</v>
-      </c>
-      <c r="H25" s="4" t="n">
+      <c r="F25" s="4" t="n">
+        <v>0.05110412975282114</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>11.03519783999736</v>
+      </c>
+      <c r="H25" s="5" t="n">
         <v>26.75</v>
       </c>
-      <c r="I25" s="5" t="n">
-        <v>0.749881599168729</v>
-      </c>
-      <c r="J25" s="2" t="n">
+      <c r="I25" s="6" t="n">
+        <v>0.7498815991687289</v>
+      </c>
+      <c r="J25" s="3" t="n">
         <v>8606</v>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="K25" s="3" t="n">
         <v>902</v>
       </c>
     </row>
@@ -1268,34 +1280,34 @@
           <t>vitamin_d</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="4" t="n">
         <v>0.7519390566538966</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="4" t="n">
         <v>0.3459019242605473</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="E26" s="4" t="n">
         <v>1.634439610946421</v>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="4" t="n">
         <v>0.03851548454774519</v>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="G26" s="4" t="n">
         <v>14.68013064253797</v>
       </c>
-      <c r="H26" s="4" t="n">
+      <c r="H26" s="5" t="n">
         <v>98.12</v>
       </c>
-      <c r="I26" s="5" t="n">
-        <v>0.01068136703040478</v>
-      </c>
-      <c r="J26" s="2" t="n">
+      <c r="I26" s="6" t="n">
+        <v>0.01068136703040477</v>
+      </c>
+      <c r="J26" s="3" t="n">
         <v>339695</v>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="K26" s="3" t="n">
         <v>4466</v>
       </c>
     </row>
@@ -1305,34 +1317,34 @@
           <t>vitamin_e</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" s="4" t="n">
         <v>0.7637612795223642</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="4" t="n">
         <v>0.5830980062410815</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="4" t="n">
         <v>1.0003000450045</v>
       </c>
-      <c r="F27" s="3" t="n">
-        <v>0.350245514116067</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>1.665492543337272</v>
-      </c>
-      <c r="H27" s="4" t="n">
+      <c r="F27" s="4" t="n">
+        <v>0.3502455141160195</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>1.665492543337498</v>
+      </c>
+      <c r="H27" s="5" t="n">
         <v>43.82</v>
       </c>
-      <c r="I27" s="5" t="n">
-        <v>0.6652833451872155</v>
-      </c>
-      <c r="J27" s="2" t="n">
+      <c r="I27" s="6" t="n">
+        <v>0.6652833451872158</v>
+      </c>
+      <c r="J27" s="3" t="n">
         <v>158299</v>
       </c>
-      <c r="K27" s="2" t="n">
+      <c r="K27" s="3" t="n">
         <v>1839</v>
       </c>
     </row>
@@ -1342,26 +1354,26 @@
           <t>vitamin_b12</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="3" t="n">
+      <c r="B28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="4" t="n">
         <v>0.7708048744499005</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="4" t="n">
         <v>0.6110819817568988</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E28" s="4" t="n">
         <v>0.990044948040641</v>
       </c>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="2" t="n">
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
+      <c r="J28" s="3" t="n">
         <v>2589</v>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="K28" s="3" t="n">
         <v>1171</v>
       </c>
     </row>
@@ -1371,34 +1383,34 @@
           <t>folic_acid</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B29" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C29" s="4" t="n">
         <v>0.7732908808107848</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="4" t="n">
         <v>0.6068340008714599</v>
       </c>
-      <c r="E29" s="3" t="n">
+      <c r="E29" s="4" t="n">
         <v>0.9854075175194142</v>
       </c>
-      <c r="F29" s="3" t="n">
-        <v>0.3516080413086398</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>1.700697128881124</v>
-      </c>
-      <c r="H29" s="4" t="n">
+      <c r="F29" s="4" t="n">
+        <v>0.3516080413085914</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>1.700697128881358</v>
+      </c>
+      <c r="H29" s="5" t="n">
         <v>63.72</v>
       </c>
-      <c r="I29" s="5" t="n">
-        <v>0.2913323489409054</v>
-      </c>
-      <c r="J29" s="2" t="n">
+      <c r="I29" s="6" t="n">
+        <v>0.2913323489409053</v>
+      </c>
+      <c r="J29" s="3" t="n">
         <v>309245</v>
       </c>
-      <c r="K29" s="2" t="n">
+      <c r="K29" s="3" t="n">
         <v>2289</v>
       </c>
     </row>
@@ -1408,28 +1420,28 @@
           <t>avocado</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="4" t="n">
         <v>0.7773224664291063</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="4" t="n">
         <v>0.5959491108750986</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E30" s="4" t="n">
         <v>1.013794275030678</v>
       </c>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr"/>
-      <c r="H30" s="4" t="n">
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="5" t="n">
         <v>20.99</v>
       </c>
-      <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="2" t="n">
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="3" t="n">
         <v>112328</v>
       </c>
-      <c r="K30" s="2" t="n">
+      <c r="K30" s="3" t="n">
         <v>1165</v>
       </c>
     </row>
@@ -1439,34 +1451,34 @@
           <t>monounsaturated_fat_mufa</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B31" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" s="4" t="n">
         <v>0.7910453344697306</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="4" t="n">
         <v>0.4113133278765659</v>
       </c>
-      <c r="E31" s="3" t="n">
+      <c r="E31" s="4" t="n">
         <v>1.521352892737078</v>
       </c>
-      <c r="F31" s="3" t="n">
-        <v>0.0002448417215769694</v>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>2555.743837921076</v>
-      </c>
-      <c r="H31" s="4" t="n">
+      <c r="F31" s="4" t="n">
+        <v>0.0002448417215368901</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>2555.743838339438</v>
+      </c>
+      <c r="H31" s="5" t="n">
         <v>88.63</v>
       </c>
-      <c r="I31" s="5" t="n">
-        <v>0.06610046025838505</v>
-      </c>
-      <c r="J31" s="2" t="n">
+      <c r="I31" s="6" t="n">
+        <v>0.06610046025838502</v>
+      </c>
+      <c r="J31" s="3" t="n">
         <v>649414</v>
       </c>
-      <c r="K31" s="2" t="n">
+      <c r="K31" s="3" t="n">
         <v>3842</v>
       </c>
     </row>
@@ -1476,34 +1488,34 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B32" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="4" t="n">
         <v>0.8285318499048928</v>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D32" s="4" t="n">
         <v>0.6515507423707737</v>
       </c>
-      <c r="E32" s="3" t="n">
+      <c r="E32" s="4" t="n">
         <v>1.053691802642768</v>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="4" t="n">
         <v>0.3820831459958125</v>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="G32" s="4" t="n">
         <v>1.796637809076109</v>
       </c>
-      <c r="H32" s="4" t="n">
+      <c r="H32" s="5" t="n">
         <v>78.58</v>
       </c>
-      <c r="I32" s="5" t="n">
-        <v>0.1380321024135174</v>
-      </c>
-      <c r="J32" s="2" t="n">
+      <c r="I32" s="6" t="n">
+        <v>0.1380321024135175</v>
+      </c>
+      <c r="J32" s="3" t="n">
         <v>799763</v>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="K32" s="3" t="n">
         <v>5469</v>
       </c>
     </row>
@@ -1513,26 +1525,26 @@
           <t>insoluble_dietary_fiber_intake</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" s="3" t="n">
+      <c r="B33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="4" t="n">
         <v>0.8303208655186842</v>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D33" s="4" t="n">
         <v>0.6705029098644103</v>
       </c>
-      <c r="E33" s="3" t="n">
+      <c r="E33" s="4" t="n">
         <v>1.029929753803904</v>
       </c>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="2" t="n">
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr"/>
+      <c r="I33" s="6" t="inlineStr"/>
+      <c r="J33" s="3" t="n">
         <v>101721</v>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="K33" s="3" t="n">
         <v>776</v>
       </c>
     </row>
@@ -1542,34 +1554,34 @@
           <t>beta_carotene</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B34" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C34" s="4" t="n">
         <v>0.8304396663075081</v>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="D34" s="4" t="n">
         <v>0.6609348544756805</v>
       </c>
-      <c r="E34" s="3" t="n">
+      <c r="E34" s="4" t="n">
         <v>1.04352040319657</v>
       </c>
-      <c r="F34" s="3" t="n">
-        <v>0.4275552528813619</v>
-      </c>
-      <c r="G34" s="3" t="n">
-        <v>1.612961213151751</v>
-      </c>
-      <c r="H34" s="4" t="n">
+      <c r="F34" s="4" t="n">
+        <v>0.4275552528813613</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>1.612961213151754</v>
+      </c>
+      <c r="H34" s="5" t="n">
         <v>58.87</v>
       </c>
-      <c r="I34" s="5" t="n">
-        <v>0.882373162497989</v>
-      </c>
-      <c r="J34" s="2" t="n">
+      <c r="I34" s="6" t="n">
+        <v>0.8823731624979892</v>
+      </c>
+      <c r="J34" s="3" t="n">
         <v>368253</v>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="K34" s="3" t="n">
         <v>2305</v>
       </c>
     </row>
@@ -1579,28 +1591,28 @@
           <t>plant_protein_intake</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B35" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C35" s="4" t="n">
         <v>0.8387018493286374</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D35" s="4" t="n">
         <v>0.7048290414313586</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="E35" s="4" t="n">
         <v>0.9981018038573761</v>
       </c>
-      <c r="F35" s="3" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="4" t="n">
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="5" t="n">
         <v>38.28</v>
       </c>
-      <c r="I35" s="5" t="inlineStr"/>
-      <c r="J35" s="2" t="n">
+      <c r="I35" s="6" t="inlineStr"/>
+      <c r="J35" s="3" t="n">
         <v>585408</v>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="K35" s="3" t="n">
         <v>2402</v>
       </c>
     </row>
@@ -1610,28 +1622,28 @@
           <t>total_dietary_fiber_intake</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B36" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C36" s="4" t="n">
         <v>0.8530816628701524</v>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="D36" s="4" t="n">
         <v>0.7636085425406669</v>
       </c>
-      <c r="E36" s="3" t="n">
+      <c r="E36" s="4" t="n">
         <v>0.9529431793814942</v>
       </c>
-      <c r="F36" s="3" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr"/>
-      <c r="H36" s="4" t="n">
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I36" s="5" t="inlineStr"/>
-      <c r="J36" s="2" t="n">
+      <c r="I36" s="6" t="inlineStr"/>
+      <c r="J36" s="3" t="n">
         <v>676447</v>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="K36" s="3" t="n">
         <v>3990</v>
       </c>
     </row>
@@ -1641,34 +1653,34 @@
           <t>alcohol</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B37" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C37" s="4" t="n">
         <v>0.8586447541387279</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D37" s="4" t="n">
         <v>0.739929771992727</v>
       </c>
-      <c r="E37" s="3" t="n">
+      <c r="E37" s="4" t="n">
         <v>0.9963068365656366</v>
       </c>
-      <c r="F37" s="3" t="n">
-        <v>0.526355059181101</v>
-      </c>
-      <c r="G37" s="3" t="n">
-        <v>1.400710035839679</v>
-      </c>
-      <c r="H37" s="4" t="n">
+      <c r="F37" s="4" t="n">
+        <v>0.5263550591747366</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>1.400710035856616</v>
+      </c>
+      <c r="H37" s="5" t="n">
         <v>84.8</v>
       </c>
-      <c r="I37" s="5" t="n">
+      <c r="I37" s="6" t="n">
         <v>0.1016499262988989</v>
       </c>
-      <c r="J37" s="2" t="n">
+      <c r="J37" s="3" t="n">
         <v>882294</v>
       </c>
-      <c r="K37" s="2" t="n">
+      <c r="K37" s="3" t="n">
         <v>8649</v>
       </c>
     </row>
@@ -1678,26 +1690,26 @@
           <t>soluble_dietary_fiber_intake</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" s="3" t="n">
-        <v>0.8602737806594901</v>
-      </c>
-      <c r="D38" s="3" t="n">
+      <c r="B38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>0.86027378065949</v>
+      </c>
+      <c r="D38" s="4" t="n">
         <v>0.6804949413246006</v>
       </c>
-      <c r="E38" s="3" t="n">
+      <c r="E38" s="4" t="n">
         <v>1.079803598340883</v>
       </c>
-      <c r="F38" s="3" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="5" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="5" t="inlineStr"/>
+      <c r="I38" s="6" t="inlineStr"/>
+      <c r="J38" s="3" t="n">
         <v>101721</v>
       </c>
-      <c r="K38" s="2" t="n">
+      <c r="K38" s="3" t="n">
         <v>776</v>
       </c>
     </row>
@@ -1707,26 +1719,26 @@
           <t>mediterranean_diet</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="3" t="n">
+      <c r="B39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="4" t="n">
         <v>0.8902226072035401</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" s="4" t="n">
         <v>0.6205359319277568</v>
       </c>
-      <c r="E39" s="3" t="n">
+      <c r="E39" s="4" t="n">
         <v>1.259255513560131</v>
       </c>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="5" t="inlineStr"/>
-      <c r="J39" s="2" t="n">
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="5" t="inlineStr"/>
+      <c r="I39" s="6" t="inlineStr"/>
+      <c r="J39" s="3" t="n">
         <v>37442</v>
       </c>
-      <c r="K39" s="2" t="n">
+      <c r="K39" s="3" t="n">
         <v>379</v>
       </c>
     </row>
@@ -1736,34 +1748,34 @@
           <t>lycopene</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B40" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="C40" s="4" t="n">
         <v>0.9475268544497669</v>
       </c>
-      <c r="D40" s="3" t="n">
+      <c r="D40" s="4" t="n">
         <v>0.9003245225862656</v>
       </c>
-      <c r="E40" s="3" t="n">
+      <c r="E40" s="4" t="n">
         <v>0.9973036417217132</v>
       </c>
-      <c r="F40" s="3" t="n">
-        <v>0.6800887710883596</v>
-      </c>
-      <c r="G40" s="3" t="n">
-        <v>1.320132279888537</v>
-      </c>
-      <c r="H40" s="4" t="n">
+      <c r="F40" s="4" t="n">
+        <v>0.6800887710837906</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>1.320132279897406</v>
+      </c>
+      <c r="H40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="5" t="n">
-        <v>0.03008236612500757</v>
-      </c>
-      <c r="J40" s="2" t="n">
+      <c r="I40" s="6" t="n">
+        <v>0.03008236612500685</v>
+      </c>
+      <c r="J40" s="3" t="n">
         <v>222792</v>
       </c>
-      <c r="K40" s="2" t="n">
+      <c r="K40" s="3" t="n">
         <v>1333</v>
       </c>
     </row>
@@ -1773,34 +1785,34 @@
           <t>tea</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B41" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C41" s="4" t="n">
         <v>0.9617507091463667</v>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D41" s="4" t="n">
         <v>0.7890701910914995</v>
       </c>
-      <c r="E41" s="3" t="n">
+      <c r="E41" s="4" t="n">
         <v>1.172337946680718</v>
       </c>
-      <c r="F41" s="3" t="n">
-        <v>0.5117552101281551</v>
-      </c>
-      <c r="G41" s="3" t="n">
+      <c r="F41" s="4" t="n">
+        <v>0.5117552101281549</v>
+      </c>
+      <c r="G41" s="4" t="n">
         <v>1.807435289836927</v>
       </c>
-      <c r="H41" s="4" t="n">
+      <c r="H41" s="5" t="n">
         <v>83.53</v>
       </c>
-      <c r="I41" s="5" t="n">
-        <v>0.02398376617759525</v>
-      </c>
-      <c r="J41" s="2" t="n">
+      <c r="I41" s="6" t="n">
+        <v>0.02398376617759524</v>
+      </c>
+      <c r="J41" s="3" t="n">
         <v>580076</v>
       </c>
-      <c r="K41" s="2" t="n">
+      <c r="K41" s="3" t="n">
         <v>9039</v>
       </c>
     </row>
@@ -1810,28 +1822,28 @@
           <t>phosphorus</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B42" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="C42" s="4" t="n">
         <v>0.9740428329225616</v>
       </c>
-      <c r="D42" s="3" t="n">
+      <c r="D42" s="4" t="n">
         <v>0.2712267749764213</v>
       </c>
-      <c r="E42" s="3" t="n">
+      <c r="E42" s="4" t="n">
         <v>3.498030164795818</v>
       </c>
-      <c r="F42" s="3" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr"/>
-      <c r="H42" s="4" t="n">
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="5" t="n">
         <v>82.45999999999999</v>
       </c>
-      <c r="I42" s="5" t="inlineStr"/>
-      <c r="J42" s="2" t="n">
+      <c r="I42" s="6" t="inlineStr"/>
+      <c r="J42" s="3" t="n">
         <v>1147</v>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="K42" s="3" t="n">
         <v>522</v>
       </c>
     </row>
@@ -1841,26 +1853,26 @@
           <t>magnesium</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="3" t="n">
+      <c r="B43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="4" t="n">
         <v>0.54113009609268</v>
       </c>
-      <c r="E43" s="3" t="n">
+      <c r="E43" s="4" t="n">
         <v>1.823130081227917</v>
       </c>
-      <c r="F43" s="3" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="5" t="inlineStr"/>
-      <c r="J43" s="2" t="n">
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="6" t="inlineStr"/>
+      <c r="J43" s="3" t="n">
         <v>574</v>
       </c>
-      <c r="K43" s="2" t="n">
+      <c r="K43" s="3" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1870,34 +1882,34 @@
           <t>vitamin_b1</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B44" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C44" s="4" t="n">
         <v>1.026135700809198</v>
       </c>
-      <c r="D44" s="3" t="n">
+      <c r="D44" s="4" t="n">
         <v>0.8760781322122511</v>
       </c>
-      <c r="E44" s="3" t="n">
+      <c r="E44" s="4" t="n">
         <v>1.201895627523871</v>
       </c>
-      <c r="F44" s="3" t="n">
-        <v>0.1861215877235061</v>
-      </c>
-      <c r="G44" s="3" t="n">
-        <v>5.657347378958566</v>
-      </c>
-      <c r="H44" s="4" t="n">
+      <c r="F44" s="4" t="n">
+        <v>0.1861215877170695</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>5.657347379154213</v>
+      </c>
+      <c r="H44" s="5" t="n">
         <v>71.67</v>
       </c>
-      <c r="I44" s="5" t="n">
-        <v>0.6179812083215517</v>
-      </c>
-      <c r="J44" s="2" t="n">
+      <c r="I44" s="6" t="n">
+        <v>0.6179812083215528</v>
+      </c>
+      <c r="J44" s="3" t="n">
         <v>575001</v>
       </c>
-      <c r="K44" s="2" t="n">
+      <c r="K44" s="3" t="n">
         <v>3737</v>
       </c>
     </row>
@@ -1907,26 +1919,26 @@
           <t>iron</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="3" t="n">
+      <c r="B45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="4" t="n">
         <v>1.049880653285851</v>
       </c>
-      <c r="D45" s="3" t="n">
+      <c r="D45" s="4" t="n">
         <v>0.9900225074278087</v>
       </c>
-      <c r="E45" s="3" t="n">
+      <c r="E45" s="4" t="n">
         <v>1.119694504834913</v>
       </c>
-      <c r="F45" s="3" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="5" t="inlineStr"/>
-      <c r="J45" s="2" t="n">
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="6" t="inlineStr"/>
+      <c r="J45" s="3" t="n">
         <v>481419</v>
       </c>
-      <c r="K45" s="2" t="n">
+      <c r="K45" s="3" t="n">
         <v>1001</v>
       </c>
     </row>
@@ -1936,28 +1948,28 @@
           <t>ultra_processed_food_intake</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
+      <c r="B46" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C46" s="4" t="n">
         <v>1.069509358657571</v>
       </c>
-      <c r="D46" s="3" t="n">
+      <c r="D46" s="4" t="n">
         <v>0.9109201832456592</v>
       </c>
-      <c r="E46" s="3" t="n">
+      <c r="E46" s="4" t="n">
         <v>1.255708556352902</v>
       </c>
-      <c r="F46" s="3" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr"/>
-      <c r="H46" s="4" t="n">
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="5" t="inlineStr"/>
-      <c r="J46" s="2" t="n">
+      <c r="I46" s="6" t="inlineStr"/>
+      <c r="J46" s="3" t="n">
         <v>647537</v>
       </c>
-      <c r="K46" s="2" t="n">
+      <c r="K46" s="3" t="n">
         <v>1906</v>
       </c>
     </row>
@@ -1967,26 +1979,26 @@
           <t>western_pattern_diet</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" s="3" t="n">
-        <v>1.089777005663734</v>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>0.8602737806594901</v>
-      </c>
-      <c r="E47" s="3" t="n">
+      <c r="B47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>1.089777005663733</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>0.86027378065949</v>
+      </c>
+      <c r="E47" s="4" t="n">
         <v>1.378808493040073</v>
       </c>
-      <c r="F47" s="3" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr"/>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="5" t="inlineStr"/>
-      <c r="J47" s="2" t="n">
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="5" t="inlineStr"/>
+      <c r="I47" s="6" t="inlineStr"/>
+      <c r="J47" s="3" t="n">
         <v>388077</v>
       </c>
-      <c r="K47" s="2" t="n">
+      <c r="K47" s="3" t="n">
         <v>822</v>
       </c>
     </row>
@@ -1996,34 +2008,34 @@
           <t>processed_meat_intake</t>
         </is>
       </c>
-      <c r="B48" s="2" t="n">
+      <c r="B48" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="C48" s="4" t="n">
         <v>1.098230227423644</v>
       </c>
-      <c r="D48" s="3" t="n">
+      <c r="D48" s="4" t="n">
         <v>0.9861961589479402</v>
       </c>
-      <c r="E48" s="3" t="n">
+      <c r="E48" s="4" t="n">
         <v>1.223113919555081</v>
       </c>
-      <c r="F48" s="3" t="n">
-        <v>0.8427431092536743</v>
-      </c>
-      <c r="G48" s="3" t="n">
-        <v>1.431171159020343</v>
-      </c>
-      <c r="H48" s="4" t="n">
+      <c r="F48" s="4" t="n">
+        <v>0.8427431092536752</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>1.431171159020342</v>
+      </c>
+      <c r="H48" s="5" t="n">
         <v>42.14</v>
       </c>
-      <c r="I48" s="5" t="n">
-        <v>0.03309532537024146</v>
-      </c>
-      <c r="J48" s="2" t="n">
+      <c r="I48" s="6" t="n">
+        <v>0.03309532537024148</v>
+      </c>
+      <c r="J48" s="3" t="n">
         <v>939835</v>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="K48" s="3" t="n">
         <v>6986</v>
       </c>
     </row>
@@ -2033,26 +2045,26 @@
           <t>sugar_sweetened_beverage_intake</t>
         </is>
       </c>
-      <c r="B49" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C49" s="3" t="n">
-        <v>1.1097224588901</v>
-      </c>
-      <c r="D49" s="3" t="n">
+      <c r="B49" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>1.109722458890099</v>
+      </c>
+      <c r="D49" s="4" t="n">
         <v>1.009977038572974</v>
       </c>
-      <c r="E49" s="3" t="n">
+      <c r="E49" s="4" t="n">
         <v>1.219390011363415</v>
       </c>
-      <c r="F49" s="3" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="5" t="inlineStr"/>
-      <c r="J49" s="2" t="n">
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
+      <c r="H49" s="5" t="inlineStr"/>
+      <c r="I49" s="6" t="inlineStr"/>
+      <c r="J49" s="3" t="n">
         <v>73024</v>
       </c>
-      <c r="K49" s="2" t="n">
+      <c r="K49" s="3" t="n">
         <v>297</v>
       </c>
     </row>
@@ -2062,28 +2074,28 @@
           <t>dietary_protein_intake</t>
         </is>
       </c>
-      <c r="B50" s="2" t="n">
+      <c r="B50" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C50" s="4" t="n">
         <v>1.117841954220713</v>
       </c>
-      <c r="D50" s="3" t="n">
+      <c r="D50" s="4" t="n">
         <v>1.012983563938329</v>
       </c>
-      <c r="E50" s="3" t="n">
+      <c r="E50" s="4" t="n">
         <v>1.233678059956743</v>
       </c>
-      <c r="F50" s="3" t="inlineStr"/>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="4" t="n">
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr"/>
+      <c r="H50" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I50" s="5" t="inlineStr"/>
-      <c r="J50" s="2" t="n">
+      <c r="I50" s="6" t="inlineStr"/>
+      <c r="J50" s="3" t="n">
         <v>585408</v>
       </c>
-      <c r="K50" s="2" t="n">
+      <c r="K50" s="3" t="n">
         <v>2402</v>
       </c>
     </row>
@@ -2093,28 +2105,28 @@
           <t>animal_protein_intake</t>
         </is>
       </c>
-      <c r="B51" s="2" t="n">
+      <c r="B51" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C51" s="4" t="n">
         <v>1.151654955944369</v>
       </c>
-      <c r="D51" s="3" t="n">
+      <c r="D51" s="4" t="n">
         <v>1.038211997081825</v>
       </c>
-      <c r="E51" s="3" t="n">
+      <c r="E51" s="4" t="n">
         <v>1.277365814492968</v>
       </c>
-      <c r="F51" s="3" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr"/>
-      <c r="H51" s="4" t="n">
+      <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr"/>
+      <c r="H51" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I51" s="5" t="inlineStr"/>
-      <c r="J51" s="2" t="n">
+      <c r="I51" s="6" t="inlineStr"/>
+      <c r="J51" s="3" t="n">
         <v>585408</v>
       </c>
-      <c r="K51" s="2" t="n">
+      <c r="K51" s="3" t="n">
         <v>2402</v>
       </c>
     </row>
@@ -2124,34 +2136,34 @@
           <t>calcium</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n">
+      <c r="B52" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C52" s="3" t="n">
+      <c r="C52" s="4" t="n">
         <v>1.169878620189307</v>
       </c>
-      <c r="D52" s="3" t="n">
+      <c r="D52" s="4" t="n">
         <v>0.8336013404157353</v>
       </c>
-      <c r="E52" s="3" t="n">
+      <c r="E52" s="4" t="n">
         <v>1.641975352073348</v>
       </c>
-      <c r="F52" s="3" t="n">
-        <v>0.02922370887848131</v>
-      </c>
-      <c r="G52" s="3" t="n">
-        <v>46.83238502227918</v>
-      </c>
-      <c r="H52" s="4" t="n">
+      <c r="F52" s="4" t="n">
+        <v>0.02922370887629698</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>46.83238502577966</v>
+      </c>
+      <c r="H52" s="5" t="n">
         <v>61.22</v>
       </c>
-      <c r="I52" s="5" t="n">
+      <c r="I52" s="6" t="n">
         <v>0.09782654651999097</v>
       </c>
-      <c r="J52" s="2" t="n">
+      <c r="J52" s="3" t="n">
         <v>493396</v>
       </c>
-      <c r="K52" s="2" t="n">
+      <c r="K52" s="3" t="n">
         <v>1881</v>
       </c>
     </row>
@@ -2161,26 +2173,26 @@
           <t>tomato</t>
         </is>
       </c>
-      <c r="B53" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" s="3" t="n">
+      <c r="B53" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4" t="n">
         <v>1.19945453907786</v>
       </c>
-      <c r="D53" s="3" t="n">
+      <c r="D53" s="4" t="n">
         <v>0.9501079967336835</v>
       </c>
-      <c r="E53" s="3" t="n">
+      <c r="E53" s="4" t="n">
         <v>1.518204486493061</v>
       </c>
-      <c r="F53" s="3" t="inlineStr"/>
-      <c r="G53" s="3" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="5" t="inlineStr"/>
-      <c r="J53" s="2" t="n">
+      <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr"/>
+      <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="6" t="inlineStr"/>
+      <c r="J53" s="3" t="n">
         <v>101683</v>
       </c>
-      <c r="K53" s="2" t="n">
+      <c r="K53" s="3" t="n">
         <v>774</v>
       </c>
     </row>
@@ -2190,34 +2202,34 @@
           <t>red_meat</t>
         </is>
       </c>
-      <c r="B54" s="2" t="n">
+      <c r="B54" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C54" s="3" t="n">
+      <c r="C54" s="4" t="n">
         <v>1.32154300883515</v>
       </c>
-      <c r="D54" s="3" t="n">
+      <c r="D54" s="4" t="n">
         <v>1.111710699877804</v>
       </c>
-      <c r="E54" s="3" t="n">
+      <c r="E54" s="4" t="n">
         <v>1.570980583701342</v>
       </c>
-      <c r="F54" s="3" t="n">
-        <v>0.7815874035063086</v>
-      </c>
-      <c r="G54" s="3" t="n">
-        <v>2.234524144537296</v>
-      </c>
-      <c r="H54" s="4" t="n">
+      <c r="F54" s="4" t="n">
+        <v>0.7815874035063085</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>2.234524144537297</v>
+      </c>
+      <c r="H54" s="5" t="n">
         <v>77.01000000000001</v>
       </c>
-      <c r="I54" s="5" t="n">
-        <v>0.01127626650555046</v>
-      </c>
-      <c r="J54" s="2" t="n">
+      <c r="I54" s="6" t="n">
+        <v>0.01127626650555044</v>
+      </c>
+      <c r="J54" s="3" t="n">
         <v>1417360</v>
       </c>
-      <c r="K54" s="2" t="n">
+      <c r="K54" s="3" t="n">
         <v>6876</v>
       </c>
     </row>
@@ -2227,26 +2239,26 @@
           <t>caffeine</t>
         </is>
       </c>
-      <c r="B55" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" s="3" t="n">
+      <c r="B55" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="4" t="n">
         <v>2.045114195119933</v>
       </c>
-      <c r="D55" s="3" t="n">
+      <c r="D55" s="4" t="n">
         <v>1.149607920243644</v>
       </c>
-      <c r="E55" s="3" t="n">
+      <c r="E55" s="4" t="n">
         <v>3.637955664073244</v>
       </c>
-      <c r="F55" s="3" t="inlineStr"/>
-      <c r="G55" s="3" t="inlineStr"/>
-      <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="5" t="inlineStr"/>
-      <c r="J55" s="2" t="n">
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
+      <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="6" t="inlineStr"/>
+      <c r="J55" s="3" t="n">
         <v>104440</v>
       </c>
-      <c r="K55" s="2" t="n">
+      <c r="K55" s="3" t="n">
         <v>206</v>
       </c>
     </row>
@@ -2256,26 +2268,26 @@
           <t>pickled_vegetables</t>
         </is>
       </c>
-      <c r="B56" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" s="3" t="n">
+      <c r="B56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="4" t="n">
         <v>3.217136946095633</v>
       </c>
-      <c r="D56" s="3" t="n">
+      <c r="D56" s="4" t="n">
         <v>1.357780842990217</v>
       </c>
-      <c r="E56" s="3" t="n">
+      <c r="E56" s="4" t="n">
         <v>7.482070687809</v>
       </c>
-      <c r="F56" s="3" t="inlineStr"/>
-      <c r="G56" s="3" t="inlineStr"/>
-      <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" s="5" t="inlineStr"/>
-      <c r="J56" s="2" t="n">
+      <c r="F56" s="4" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="6" t="inlineStr"/>
+      <c r="J56" s="3" t="n">
         <v>260</v>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="K56" s="3" t="n">
         <v>130</v>
       </c>
     </row>
@@ -2285,26 +2297,26 @@
           <t>vegetable_and_seed_oil_intake</t>
         </is>
       </c>
-      <c r="B57" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" s="3" t="n">
+      <c r="B57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="4" t="n">
         <v>3.431519625226634</v>
       </c>
-      <c r="D57" s="3" t="n">
+      <c r="D57" s="4" t="n">
         <v>1.684722438489189</v>
       </c>
-      <c r="E57" s="3" t="n">
+      <c r="E57" s="4" t="n">
         <v>6.946365883186642</v>
       </c>
-      <c r="F57" s="3" t="inlineStr"/>
-      <c r="G57" s="3" t="inlineStr"/>
-      <c r="H57" s="4" t="inlineStr"/>
-      <c r="I57" s="5" t="inlineStr"/>
-      <c r="J57" s="2" t="n">
+      <c r="F57" s="4" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr"/>
+      <c r="I57" s="6" t="inlineStr"/>
+      <c r="J57" s="3" t="n">
         <v>405</v>
       </c>
-      <c r="K57" s="2" t="n">
+      <c r="K57" s="3" t="n">
         <v>113</v>
       </c>
     </row>
@@ -2314,28 +2326,28 @@
           <t>eggs</t>
         </is>
       </c>
-      <c r="B58" s="2" t="n">
+      <c r="B58" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C58" s="3" t="n">
+      <c r="C58" s="4" t="n">
         <v>3.857811292537815</v>
       </c>
-      <c r="D58" s="3" t="n">
+      <c r="D58" s="4" t="n">
         <v>2.646928735129925</v>
       </c>
-      <c r="E58" s="3" t="n">
+      <c r="E58" s="4" t="n">
         <v>5.622632665288498</v>
       </c>
-      <c r="F58" s="3" t="inlineStr"/>
-      <c r="G58" s="3" t="inlineStr"/>
-      <c r="H58" s="4" t="n">
+      <c r="F58" s="4" t="inlineStr"/>
+      <c r="G58" s="4" t="inlineStr"/>
+      <c r="H58" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I58" s="5" t="inlineStr"/>
-      <c r="J58" s="2" t="n">
+      <c r="I58" s="6" t="inlineStr"/>
+      <c r="J58" s="3" t="n">
         <v>1995</v>
       </c>
-      <c r="K58" s="2" t="n">
+      <c r="K58" s="3" t="n">
         <v>355</v>
       </c>
     </row>
@@ -2345,26 +2357,26 @@
           <t>soy</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C59" s="3" t="n">
+      <c r="B59" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="4" t="n">
         <v>4.61</v>
       </c>
-      <c r="D59" s="3" t="n">
+      <c r="D59" s="4" t="n">
         <v>1.57</v>
       </c>
-      <c r="E59" s="3" t="n">
+      <c r="E59" s="4" t="n">
         <v>13.51</v>
       </c>
-      <c r="F59" s="3" t="inlineStr"/>
-      <c r="G59" s="3" t="inlineStr"/>
-      <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="5" t="inlineStr"/>
-      <c r="J59" s="2" t="n">
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr"/>
+      <c r="H59" s="5" t="inlineStr"/>
+      <c r="I59" s="6" t="inlineStr"/>
+      <c r="J59" s="3" t="n">
         <v>18244</v>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="K59" s="3" t="n">
         <v>61</v>
       </c>
     </row>
@@ -2374,26 +2386,26 @@
           <t>anti_inflammatory_diet</t>
         </is>
       </c>
-      <c r="B60" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C60" s="3" t="n">
+      <c r="B60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="4" t="n">
         <v>5.609539624201962</v>
       </c>
-      <c r="D60" s="3" t="n">
+      <c r="D60" s="4" t="n">
         <v>1.456957290394739</v>
       </c>
-      <c r="E60" s="3" t="n">
+      <c r="E60" s="4" t="n">
         <v>20.44949521459941</v>
       </c>
-      <c r="F60" s="3" t="inlineStr"/>
-      <c r="G60" s="3" t="inlineStr"/>
-      <c r="H60" s="4" t="inlineStr"/>
-      <c r="I60" s="5" t="inlineStr"/>
-      <c r="J60" s="2" t="n">
+      <c r="F60" s="4" t="inlineStr"/>
+      <c r="G60" s="4" t="inlineStr"/>
+      <c r="H60" s="5" t="inlineStr"/>
+      <c r="I60" s="6" t="inlineStr"/>
+      <c r="J60" s="3" t="n">
         <v>199</v>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="K60" s="3" t="n">
         <v>95</v>
       </c>
     </row>

</xml_diff>